<commit_message>
#25 Peripheral Added in BOM
</commit_message>
<xml_diff>
--- a/Design Files/Ezlo-Radar-Sensor-v2.0-Advance/BOM/Client_BOM.xlsx
+++ b/Design Files/Ezlo-Radar-Sensor-v2.0-Advance/BOM/Client_BOM.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\ezlo-thermostat\Design Files\Ezlo-Radar-Sensor-v2.0-Advance\Project Outputs for Ezlo-Radar-Sensor-v2.0-Advance\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\ezlo-thermostat\Design Files\Ezlo-Radar-Sensor-v2.0-Advance\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="85">
   <si>
     <t>#</t>
   </si>
@@ -267,10 +267,13 @@
     <t>peripheral</t>
   </si>
   <si>
-    <t xml:space="preserve">Flexible Cable </t>
-  </si>
-  <si>
-    <t>Length Required</t>
+    <t>KH-FFC-A0.5-15P-120MM</t>
+  </si>
+  <si>
+    <t>15 0.5mm Same Side 120mm P=0.5mm FFC/FPC Connect Cables ROHS</t>
+  </si>
+  <si>
+    <t>Shenzhen Kinghelm Elec</t>
   </si>
 </sst>
 </file>
@@ -589,14 +592,14 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -909,9 +912,9 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -952,7 +955,7 @@
         <f>ROW(B3) - ROW($B$2)</f>
         <v>1</v>
       </c>
-      <c r="C3" s="25" t="s">
+      <c r="C3" s="24" t="s">
         <v>2</v>
       </c>
       <c r="D3" s="15" t="s">
@@ -984,7 +987,7 @@
         <f t="shared" ref="B4:B14" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
-      <c r="C4" s="25" t="s">
+      <c r="C4" s="24" t="s">
         <v>2</v>
       </c>
       <c r="D4" s="17" t="s">
@@ -1016,7 +1019,7 @@
         <f>ROW(B5) - ROW($B$2)</f>
         <v>3</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="C5" s="24" t="s">
         <v>2</v>
       </c>
       <c r="D5" s="15" t="s">
@@ -1048,7 +1051,7 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="C6" s="24" t="s">
         <v>2</v>
       </c>
       <c r="D6" s="17" t="s">
@@ -1080,7 +1083,7 @@
         <f>ROW(B7) - ROW($B$2)</f>
         <v>5</v>
       </c>
-      <c r="C7" s="25" t="s">
+      <c r="C7" s="24" t="s">
         <v>2</v>
       </c>
       <c r="D7" s="15" t="s">
@@ -1112,7 +1115,7 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C8" s="25" t="s">
+      <c r="C8" s="24" t="s">
         <v>2</v>
       </c>
       <c r="D8" s="17" t="s">
@@ -1144,7 +1147,7 @@
         <f>ROW(B9) - ROW($B$2)</f>
         <v>7</v>
       </c>
-      <c r="C9" s="26" t="s">
+      <c r="C9" s="25" t="s">
         <v>3</v>
       </c>
       <c r="D9" s="15" t="s">
@@ -1176,7 +1179,7 @@
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C10" s="25" t="s">
+      <c r="C10" s="24" t="s">
         <v>4</v>
       </c>
       <c r="D10" s="17" t="s">
@@ -1208,7 +1211,7 @@
         <f>ROW(B11) - ROW($B$2)</f>
         <v>9</v>
       </c>
-      <c r="C11" s="26" t="s">
+      <c r="C11" s="25" t="s">
         <v>5</v>
       </c>
       <c r="D11" s="15" t="s">
@@ -1240,7 +1243,7 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C12" s="25" t="s">
+      <c r="C12" s="24" t="s">
         <v>6</v>
       </c>
       <c r="D12" s="17" t="s">
@@ -1272,7 +1275,7 @@
         <f>ROW(B13) - ROW($B$2)</f>
         <v>11</v>
       </c>
-      <c r="C13" s="26" t="s">
+      <c r="C13" s="25" t="s">
         <v>7</v>
       </c>
       <c r="D13" s="15" t="s">
@@ -1304,7 +1307,7 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C14" s="25" t="s">
+      <c r="C14" s="24" t="s">
         <v>7</v>
       </c>
       <c r="D14" s="17" t="s">
@@ -1336,7 +1339,7 @@
         <f>ROW(B15) - ROW($B$2)</f>
         <v>13</v>
       </c>
-      <c r="C15" s="26" t="s">
+      <c r="C15" s="25" t="s">
         <v>8</v>
       </c>
       <c r="D15" s="15" t="s">
@@ -1362,20 +1365,20 @@
       </c>
       <c r="K15" s="15"/>
     </row>
-    <row r="16" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="23">
         <f t="shared" ref="B16" si="1">ROW(B16) - ROW($B$2)</f>
         <v>14</v>
       </c>
-      <c r="C16" s="26" t="s">
+      <c r="C16" s="25" t="s">
         <v>81</v>
       </c>
       <c r="D16" s="15" t="s">
         <v>80</v>
       </c>
       <c r="E16" s="15" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F16" s="15" t="s">
         <v>80</v>
@@ -1384,15 +1387,15 @@
         <v>82</v>
       </c>
       <c r="H16" s="15" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="I16" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="J16" s="15"/>
-      <c r="K16" s="15" t="s">
-        <v>83</v>
-      </c>
+      <c r="J16" s="15">
+        <v>1</v>
+      </c>
+      <c r="K16" s="15"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>

</xml_diff>